<commit_message>
25.11 fb clinical template (#1699)
* Modified program to include Non pregnant selection item.

* Modified program to include Non pregnant selection item.

* Modified Clinical upload template.

* Modified Clinical upload template.

* Modified Clinical upload template.

* Modified Clinical upload template.

* Modified Clinical upload template.

---------

Co-authored-by: blasar <blasar@ohsu.eddu>
</commit_message>
<xml_diff>
--- a/onprc_ehr/resources/web/onprc_ehr/templates/ClinicalProcessingTemplate_TPR_Master.xlsx
+++ b/onprc_ehr/resources/web/onprc_ehr/templates/ClinicalProcessingTemplate_TPR_Master.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10419"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\XML_Project\Heather_Panaro\ClinicalProcessing_TPR\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/tmp/blasarVolumes/blasar/XML_Project/Heather_Panaro/ClinicalProcessing_TPR/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47CE8D58-1FD1-48A3-AABF-154712485536}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3E27658-A070-9142-B0FA-9CFA70119565}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="V0mH21jSP57WeMvfm2GZf/CFapX9PbyX3c7CLbaowv65HEOfZYZks22oton1PO1KhMKfP/Yy+b48PowhVvmdMw==" workbookSaltValue="7RYukLmSAngqyTzJhGnEpg==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="2730" yWindow="1770" windowWidth="25170" windowHeight="13710" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3420" yWindow="3220" windowWidth="29580" windowHeight="15040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ClinProcessing Entry Template" sheetId="6" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="174">
   <si>
     <t>Id</t>
   </si>
@@ -154,24 +154,12 @@
     <t>cullin</t>
   </si>
   <si>
-    <t>Heather Sidener</t>
-  </si>
-  <si>
-    <t>sidener</t>
-  </si>
-  <si>
     <t>Jeff Stanton</t>
   </si>
   <si>
     <t>stantoje</t>
   </si>
   <si>
-    <t>Kamm Prongay</t>
-  </si>
-  <si>
-    <t>prongayk</t>
-  </si>
-  <si>
     <t>Rhonda MacAllister</t>
   </si>
   <si>
@@ -229,9 +217,6 @@
     <t>Applies to Preg column with "1, 2, or 3" value</t>
   </si>
   <si>
-    <t>Preg Qualifier</t>
-  </si>
-  <si>
     <t>Applies to Preg column with "3" value</t>
   </si>
   <si>
@@ -536,13 +521,52 @@
   </si>
   <si>
     <t>Turgor Observation</t>
+  </si>
+  <si>
+    <t>Applies to Preg column with "No" value</t>
+  </si>
+  <si>
+    <t>NON PREGNANT STATE (F-30980)</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Drew Martin</t>
+  </si>
+  <si>
+    <t>martilau</t>
+  </si>
+  <si>
+    <t>Eden Doh</t>
+  </si>
+  <si>
+    <t>dohe</t>
+  </si>
+  <si>
+    <t>Joshua Taylor</t>
+  </si>
+  <si>
+    <t>tayljosh</t>
+  </si>
+  <si>
+    <t>Kendall Lewis</t>
+  </si>
+  <si>
+    <t>lewisken</t>
+  </si>
+  <si>
+    <t>Monica Stroyer</t>
+  </si>
+  <si>
+    <t>shroyer</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -598,6 +622,19 @@
       <name val="JetBrains Mono"/>
       <family val="3"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -639,7 +676,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -733,6 +770,8 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1040,25 +1079,25 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet3"/>
-  <dimension ref="A1:P609"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <dimension ref="A1:P699"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="22.85546875" style="12" customWidth="1"/>
-    <col min="2" max="2" width="52.140625" style="11" customWidth="1"/>
-    <col min="3" max="3" width="39.5703125" style="11" customWidth="1"/>
-    <col min="4" max="4" width="7.5703125" style="11" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.7109375" style="11" customWidth="1"/>
-    <col min="6" max="6" width="7.28515625" style="11" customWidth="1"/>
-    <col min="7" max="7" width="8.28515625" style="11" customWidth="1"/>
-    <col min="8" max="11" width="6.28515625" style="11" customWidth="1"/>
-    <col min="12" max="12" width="4.140625" style="11" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="101.85546875" style="11" customWidth="1"/>
-    <col min="14" max="14" width="11.85546875" style="11" customWidth="1"/>
-    <col min="15" max="15" width="9.140625" style="27"/>
-    <col min="16" max="16384" width="9.140625" style="11"/>
+    <col min="1" max="1" width="22.83203125" style="12" customWidth="1"/>
+    <col min="2" max="2" width="52.1640625" style="11" customWidth="1"/>
+    <col min="3" max="3" width="39.5" style="11" customWidth="1"/>
+    <col min="4" max="4" width="7.5" style="11" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.6640625" style="11" customWidth="1"/>
+    <col min="6" max="6" width="7.33203125" style="11" customWidth="1"/>
+    <col min="7" max="7" width="8.33203125" style="11" customWidth="1"/>
+    <col min="8" max="11" width="6.33203125" style="11" customWidth="1"/>
+    <col min="12" max="12" width="4.1640625" style="11" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="101.83203125" style="11" customWidth="1"/>
+    <col min="14" max="14" width="11.83203125" style="11" customWidth="1"/>
+    <col min="15" max="15" width="9.1640625" style="27"/>
+    <col min="16" max="16384" width="9.1640625" style="11"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="18.75">
+    <row r="1" spans="1:13" ht="19">
       <c r="A1" s="10" t="s">
         <v>12</v>
       </c>
@@ -1079,20 +1118,20 @@
         <v>11</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="C5" s="11" t="str">
+        <v>46</v>
+      </c>
+      <c r="C5" s="11" t="e">
         <f>VLOOKUP(B5,'Drop-down lists'!A2:B12,2,FALSE)</f>
-        <v xml:space="preserve"> </v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="14.25" customHeight="1">
       <c r="A6" s="13"/>
       <c r="B6" s="15"/>
     </row>
-    <row r="7" spans="1:13">
+    <row r="7" spans="1:13" hidden="1">
       <c r="A7" s="16" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="B7" s="17"/>
       <c r="C7" s="18"/>
@@ -1107,62 +1146,62 @@
       <c r="L7" s="18"/>
       <c r="M7" s="18"/>
     </row>
-    <row r="8" spans="1:13">
+    <row r="8" spans="1:13" hidden="1">
       <c r="A8" s="12" t="s">
         <v>0</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" hidden="1">
       <c r="A9" s="12" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" hidden="1">
       <c r="A10" s="12" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" hidden="1">
       <c r="A11" s="12" t="s">
         <v>15</v>
       </c>
       <c r="B11" s="19" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" hidden="1">
       <c r="A12" s="12" t="s">
         <v>16</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="C12" s="15" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" hidden="1">
       <c r="A13" s="12" t="s">
         <v>14</v>
       </c>
@@ -1170,38 +1209,38 @@
         <v>13</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" hidden="1">
       <c r="A14" s="12" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" hidden="1">
       <c r="A15" s="12" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="C15" s="15" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" hidden="1">
       <c r="B16" s="3"/>
       <c r="D16" s="15"/>
     </row>
-    <row r="17" spans="1:13">
+    <row r="17" spans="1:13" hidden="1">
       <c r="A17" s="16" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="B17" s="20"/>
       <c r="C17" s="18"/>
@@ -1216,158 +1255,158 @@
       <c r="L17" s="18"/>
       <c r="M17" s="18"/>
     </row>
-    <row r="18" spans="1:13">
+    <row r="18" spans="1:13" hidden="1">
       <c r="A18" s="12" t="s">
         <v>0</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="C18" s="15" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="19" spans="1:13">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" hidden="1">
       <c r="A19" s="12" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C19" s="15" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="20" spans="1:13">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" hidden="1">
       <c r="A20" s="12" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C20" s="15" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="21" spans="1:13">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" hidden="1">
       <c r="A21" s="12" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>17</v>
       </c>
       <c r="C21" s="15" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="22" spans="1:13">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" hidden="1">
       <c r="A22" s="12" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="C22" s="15" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="H22" s="15"/>
     </row>
-    <row r="23" spans="1:13">
+    <row r="23" spans="1:13" hidden="1">
       <c r="A23" s="12" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C23" s="15" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="H23" s="15"/>
     </row>
-    <row r="24" spans="1:13">
+    <row r="24" spans="1:13" hidden="1">
       <c r="A24" s="12" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C24" s="15" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="H24" s="15"/>
     </row>
-    <row r="25" spans="1:13">
+    <row r="25" spans="1:13" hidden="1">
       <c r="A25" s="12" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>18</v>
       </c>
       <c r="C25" s="15" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="H25" s="15"/>
     </row>
-    <row r="26" spans="1:13">
+    <row r="26" spans="1:13" hidden="1">
       <c r="A26" s="12" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>19</v>
       </c>
       <c r="C26" s="15" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="27" spans="1:13">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" hidden="1">
       <c r="A27" s="12" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C27" s="15" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="28" spans="1:13">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" hidden="1">
       <c r="A28" s="12" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="C28" s="15" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="29" spans="1:13">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" hidden="1">
       <c r="A29" s="12" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C29" s="15" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="30" spans="1:13">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" hidden="1">
       <c r="A30" s="12" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="D30" s="15"/>
     </row>
-    <row r="31" spans="1:13">
+    <row r="31" spans="1:13" hidden="1">
       <c r="B31" s="3"/>
       <c r="D31" s="15"/>
     </row>
-    <row r="32" spans="1:13">
+    <row r="32" spans="1:13" hidden="1">
       <c r="A32" s="16" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="B32" s="20"/>
       <c r="C32" s="18"/>
@@ -1382,471 +1421,471 @@
       <c r="L32" s="18"/>
       <c r="M32" s="18"/>
     </row>
-    <row r="33" spans="1:3">
+    <row r="33" spans="1:3" hidden="1">
       <c r="A33" s="12" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="B33" s="15" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="C33" s="15" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" hidden="1">
       <c r="A34" s="12" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="B34" s="15" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C34" s="15" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" hidden="1">
       <c r="A35" s="12" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="B35" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C35" s="15" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" hidden="1">
+      <c r="A36" s="12" t="s">
         <v>91</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3">
-      <c r="A36" s="12" t="s">
-        <v>96</v>
       </c>
       <c r="B36" s="3" t="s">
         <v>21</v>
       </c>
       <c r="C36" s="15" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" hidden="1">
       <c r="A37" s="12" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="C37" s="15" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" hidden="1">
       <c r="A38" s="12" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="B38" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C38" s="15" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" hidden="1">
+      <c r="A39" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="C39" s="15" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" hidden="1">
+      <c r="A40" s="15" t="s">
+        <v>85</v>
+      </c>
+      <c r="B40" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="C40" s="15" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" hidden="1">
+      <c r="A41" s="15" t="s">
+        <v>84</v>
+      </c>
+      <c r="B41" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="C38" s="15" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3">
-      <c r="A39" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="B39" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="C39" s="15" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3">
-      <c r="A40" s="15" t="s">
-        <v>90</v>
-      </c>
-      <c r="B40" s="15" t="s">
-        <v>60</v>
-      </c>
-      <c r="C40" s="15" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3">
-      <c r="A41" s="15" t="s">
-        <v>89</v>
-      </c>
-      <c r="B41" s="15" t="s">
-        <v>58</v>
-      </c>
       <c r="C41" s="15" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" hidden="1">
       <c r="A42" s="12" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="B42" s="3" t="s">
         <v>20</v>
       </c>
       <c r="C42" s="15" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" hidden="1">
+      <c r="A43" s="12" t="s">
         <v>82</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3">
-      <c r="A43" s="12" t="s">
-        <v>87</v>
       </c>
       <c r="B43" s="3" t="s">
         <v>21</v>
       </c>
       <c r="C43" s="15" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" hidden="1">
       <c r="A44" s="12" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="C44" s="15" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" hidden="1">
       <c r="A45" s="12" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="B45" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C45" s="15" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" hidden="1">
+      <c r="A46" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="C46" s="15" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" hidden="1">
+      <c r="A47" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="B47" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="C47" s="15" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" hidden="1">
+      <c r="A48" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="B48" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="C45" s="15" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3">
-      <c r="A46" s="12" t="s">
-        <v>83</v>
-      </c>
-      <c r="B46" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="C46" s="15" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3">
-      <c r="A47" s="12" t="s">
-        <v>81</v>
-      </c>
-      <c r="B47" s="15" t="s">
-        <v>60</v>
-      </c>
-      <c r="C47" s="15" t="s">
+      <c r="C48" s="15" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" hidden="1">
+      <c r="A49" s="12" t="s">
         <v>74</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3">
-      <c r="A48" s="12" t="s">
-        <v>80</v>
-      </c>
-      <c r="B48" s="15" t="s">
-        <v>58</v>
-      </c>
-      <c r="C48" s="15" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3">
-      <c r="A49" s="12" t="s">
-        <v>79</v>
       </c>
       <c r="B49" s="3" t="s">
         <v>22</v>
       </c>
       <c r="C49" s="15" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" hidden="1">
       <c r="A50" s="12" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="B50" s="3" t="s">
         <v>21</v>
       </c>
       <c r="C50" s="15" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" hidden="1">
       <c r="A51" s="12" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="B51" s="3" t="s">
         <v>23</v>
       </c>
       <c r="C51" s="15" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" hidden="1">
       <c r="A52" s="12" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="B52" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C52" s="15" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" hidden="1">
+      <c r="A53" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="C53" s="15" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" hidden="1">
+      <c r="A54" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="B54" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="C54" s="15" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" hidden="1">
+      <c r="A55" s="15" t="s">
+        <v>120</v>
+      </c>
+      <c r="B55" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="C52" s="15" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3">
-      <c r="A53" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="B53" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="C53" s="15" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3">
-      <c r="A54" s="15" t="s">
-        <v>124</v>
-      </c>
-      <c r="B54" s="15" t="s">
-        <v>60</v>
-      </c>
-      <c r="C54" s="15" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3">
-      <c r="A55" s="15" t="s">
-        <v>125</v>
-      </c>
-      <c r="B55" s="15" t="s">
-        <v>58</v>
-      </c>
       <c r="C55" s="15" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" hidden="1">
       <c r="A56" s="12" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="C56" s="15" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" hidden="1">
       <c r="A57" s="12" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="B57" s="3" t="s">
         <v>21</v>
       </c>
       <c r="C57" s="15" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" hidden="1">
       <c r="A58" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="B58" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="C58" s="15" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" hidden="1">
+      <c r="A59" s="12" t="s">
+        <v>124</v>
+      </c>
+      <c r="B59" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C59" s="15" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" hidden="1">
+      <c r="A60" s="12" t="s">
+        <v>125</v>
+      </c>
+      <c r="B60" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="C60" s="15" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" hidden="1">
+      <c r="A61" s="15" t="s">
+        <v>126</v>
+      </c>
+      <c r="B61" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="C61" s="15" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" hidden="1">
+      <c r="A62" s="15" t="s">
+        <v>127</v>
+      </c>
+      <c r="B62" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="C62" s="15" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" hidden="1">
+      <c r="A63" s="12" t="s">
         <v>128</v>
       </c>
-      <c r="B58" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="C58" s="15" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3">
-      <c r="A59" s="12" t="s">
+      <c r="B63" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="C63" s="15" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" hidden="1">
+      <c r="A64" s="12" t="s">
         <v>129</v>
-      </c>
-      <c r="B59" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="C59" s="15" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3">
-      <c r="A60" s="12" t="s">
-        <v>130</v>
-      </c>
-      <c r="B60" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="C60" s="15" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3">
-      <c r="A61" s="15" t="s">
-        <v>131</v>
-      </c>
-      <c r="B61" s="15" t="s">
-        <v>60</v>
-      </c>
-      <c r="C61" s="15" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3">
-      <c r="A62" s="15" t="s">
-        <v>132</v>
-      </c>
-      <c r="B62" s="15" t="s">
-        <v>58</v>
-      </c>
-      <c r="C62" s="15" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3">
-      <c r="A63" s="12" t="s">
-        <v>133</v>
-      </c>
-      <c r="B63" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="C63" s="15" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3">
-      <c r="A64" s="12" t="s">
-        <v>134</v>
       </c>
       <c r="B64" s="3" t="s">
         <v>21</v>
       </c>
       <c r="C64" s="15" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="65" spans="1:13" hidden="1">
+      <c r="A65" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="B65" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="C65" s="15" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="66" spans="1:13" hidden="1">
+      <c r="A66" s="12" t="s">
+        <v>132</v>
+      </c>
+      <c r="B66" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C66" s="15" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="67" spans="1:13" hidden="1">
+      <c r="A67" s="12" t="s">
+        <v>133</v>
+      </c>
+      <c r="B67" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="C67" s="15" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="68" spans="1:13" hidden="1">
+      <c r="A68" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="B68" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="C68" s="15" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="69" spans="1:13" hidden="1">
+      <c r="A69" s="15" t="s">
+        <v>137</v>
+      </c>
+      <c r="B69" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="C69" s="15" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="70" spans="1:13" hidden="1">
+      <c r="A70" s="12" t="s">
+        <v>138</v>
+      </c>
+      <c r="B70" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="C70" s="15" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="71" spans="1:13" hidden="1">
+      <c r="A71" s="12" t="s">
         <v>139</v>
-      </c>
-    </row>
-    <row r="65" spans="1:13">
-      <c r="A65" s="12" t="s">
-        <v>135</v>
-      </c>
-      <c r="B65" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="C65" s="15" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="66" spans="1:13">
-      <c r="A66" s="12" t="s">
-        <v>137</v>
-      </c>
-      <c r="B66" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="C66" s="15" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="67" spans="1:13">
-      <c r="A67" s="12" t="s">
-        <v>138</v>
-      </c>
-      <c r="B67" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="C67" s="15" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="68" spans="1:13">
-      <c r="A68" s="15" t="s">
-        <v>141</v>
-      </c>
-      <c r="B68" s="15" t="s">
-        <v>60</v>
-      </c>
-      <c r="C68" s="15" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="69" spans="1:13">
-      <c r="A69" s="15" t="s">
-        <v>142</v>
-      </c>
-      <c r="B69" s="15" t="s">
-        <v>58</v>
-      </c>
-      <c r="C69" s="15" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="70" spans="1:13">
-      <c r="A70" s="12" t="s">
-        <v>143</v>
-      </c>
-      <c r="B70" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="C70" s="15" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="71" spans="1:13">
-      <c r="A71" s="12" t="s">
-        <v>144</v>
       </c>
       <c r="B71" s="3" t="s">
         <v>21</v>
       </c>
       <c r="C71" s="15" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="72" spans="1:13">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="72" spans="1:13" hidden="1">
       <c r="A72" s="12" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="C72" s="15" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="73" spans="1:13">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="73" spans="1:13" hidden="1">
       <c r="A73" s="12" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C73" s="15" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="74" spans="1:13">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="74" spans="1:13" hidden="1">
       <c r="A74" s="12" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="C74" s="15" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="75" spans="1:13">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="75" spans="1:13" hidden="1">
       <c r="A75" s="21" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="B75" s="22"/>
       <c r="C75" s="23"/>
@@ -1861,198 +1900,198 @@
       <c r="L75" s="23"/>
       <c r="M75" s="23"/>
     </row>
-    <row r="76" spans="1:13">
+    <row r="76" spans="1:13" hidden="1">
       <c r="A76" s="12" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="B76" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="C76" s="15" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="77" spans="1:13" hidden="1">
+      <c r="A77" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="B77" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="C77" s="15" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="78" spans="1:13" hidden="1">
+      <c r="A78" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="B78" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="C78" s="15" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="79" spans="1:13" hidden="1">
+      <c r="A79" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="B79" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="C79" s="15" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="80" spans="1:13" hidden="1">
+      <c r="A80" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="B80" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="C76" s="15" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="77" spans="1:13">
-      <c r="A77" s="12" t="s">
-        <v>71</v>
-      </c>
-      <c r="B77" s="15" t="s">
-        <v>58</v>
-      </c>
-      <c r="C77" s="15" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="78" spans="1:13">
-      <c r="A78" s="12" t="s">
-        <v>66</v>
-      </c>
-      <c r="B78" s="15" t="s">
-        <v>70</v>
-      </c>
-      <c r="C78" s="15" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="79" spans="1:13">
-      <c r="A79" s="12" t="s">
-        <v>66</v>
-      </c>
-      <c r="B79" s="15" t="s">
-        <v>68</v>
-      </c>
-      <c r="C79" s="15" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="80" spans="1:13">
-      <c r="A80" s="12" t="s">
-        <v>66</v>
-      </c>
-      <c r="B80" s="3" t="s">
-        <v>65</v>
-      </c>
       <c r="C80" s="15" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="81" spans="1:16">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="81" spans="1:16" hidden="1">
       <c r="A81" s="12" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B81" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="C81" s="15" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="82" spans="1:16" hidden="1">
+      <c r="A82" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="B82" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="C82" s="15" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="83" spans="1:16" hidden="1">
+      <c r="A83" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="B83" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="C81" s="15" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="82" spans="1:16">
-      <c r="A82" s="12" t="s">
-        <v>61</v>
-      </c>
-      <c r="B82" s="15" t="s">
-        <v>60</v>
-      </c>
-      <c r="C82" s="15" t="s">
+      <c r="C83" s="15" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="84" spans="1:16" hidden="1">
+      <c r="A84" s="12" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="83" spans="1:16">
-      <c r="A83" s="12" t="s">
-        <v>59</v>
-      </c>
-      <c r="B83" s="15" t="s">
-        <v>58</v>
-      </c>
-      <c r="C83" s="15" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="84" spans="1:16">
-      <c r="A84" s="12" t="s">
-        <v>57</v>
-      </c>
       <c r="B84" s="3" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C84" s="15" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="85" spans="1:16">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="85" spans="1:16" hidden="1">
       <c r="A85" s="12" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="B85" s="3" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C85" s="15" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="86" spans="1:16">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="86" spans="1:16" hidden="1">
       <c r="A86" s="12" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="B86" s="3" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="C86" s="15"/>
     </row>
-    <row r="87" spans="1:16">
+    <row r="87" spans="1:16" hidden="1">
       <c r="A87" s="12" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="B87" s="3" t="s">
         <v>21</v>
       </c>
       <c r="C87" s="15"/>
     </row>
-    <row r="88" spans="1:16">
+    <row r="88" spans="1:16" hidden="1">
       <c r="A88" s="12" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="B88" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="C88" s="15"/>
+    </row>
+    <row r="89" spans="1:16" hidden="1">
+      <c r="A89" s="12" t="s">
         <v>155</v>
       </c>
-      <c r="C88" s="15"/>
-    </row>
-    <row r="89" spans="1:16">
-      <c r="A89" s="12" t="s">
-        <v>160</v>
-      </c>
       <c r="B89" s="3" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="C89" s="15"/>
     </row>
-    <row r="90" spans="1:16">
+    <row r="90" spans="1:16" hidden="1">
       <c r="A90" s="13" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="B90" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D90" s="15"/>
     </row>
-    <row r="91" spans="1:16">
+    <row r="91" spans="1:16" hidden="1">
       <c r="A91" s="13" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="B91" s="29" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="D91" s="15"/>
     </row>
-    <row r="92" spans="1:16">
+    <row r="92" spans="1:16" hidden="1">
       <c r="A92" s="13" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="B92" s="29" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="D92" s="15"/>
     </row>
-    <row r="93" spans="1:16">
+    <row r="93" spans="1:16" hidden="1">
       <c r="A93" s="13" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="B93" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D93" s="15"/>
     </row>
-    <row r="94" spans="1:16">
+    <row r="94" spans="1:16" hidden="1">
       <c r="A94" s="13" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="B94" s="3" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="D94" s="15"/>
     </row>
-    <row r="95" spans="1:16">
+    <row r="95" spans="1:16" hidden="1">
       <c r="A95" s="13"/>
       <c r="B95" s="3"/>
       <c r="D95" s="15"/>
@@ -2071,13 +2110,13 @@
         <v>3</v>
       </c>
       <c r="E96" s="25" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="F96" s="25" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="G96" s="25" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="H96" s="25" t="s">
         <v>4</v>
@@ -2098,13 +2137,13 @@
         <v>5</v>
       </c>
       <c r="N96" s="11" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="O96" s="27" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="P96" s="11" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
     </row>
     <row r="97" spans="1:15" s="7" customFormat="1">
@@ -4707,89 +4746,359 @@
       <c r="H597" s="8"/>
       <c r="O597" s="28"/>
     </row>
+    <row r="598" spans="1:15">
+      <c r="K598" s="7"/>
+    </row>
     <row r="599" spans="1:15">
       <c r="E599" s="15"/>
       <c r="F599" s="15"/>
       <c r="G599" s="15"/>
-      <c r="K599" s="15"/>
+      <c r="K599" s="7"/>
       <c r="L599" s="15"/>
     </row>
     <row r="600" spans="1:15">
       <c r="E600" s="15"/>
       <c r="F600" s="15"/>
       <c r="G600" s="15"/>
-      <c r="K600" s="15"/>
+      <c r="K600" s="7"/>
       <c r="L600" s="15"/>
     </row>
     <row r="601" spans="1:15">
       <c r="E601" s="15"/>
       <c r="F601" s="15"/>
       <c r="G601" s="15"/>
-      <c r="K601" s="15"/>
+      <c r="K601" s="7"/>
       <c r="L601" s="15"/>
     </row>
     <row r="602" spans="1:15">
       <c r="E602" s="15"/>
       <c r="F602" s="15"/>
       <c r="G602" s="15"/>
-      <c r="K602" s="15"/>
+      <c r="K602" s="7"/>
       <c r="L602" s="15"/>
     </row>
     <row r="603" spans="1:15">
       <c r="E603" s="15"/>
       <c r="F603" s="15"/>
       <c r="G603" s="15"/>
-      <c r="K603" s="15"/>
+      <c r="K603" s="7"/>
       <c r="L603" s="15"/>
     </row>
     <row r="604" spans="1:15">
       <c r="E604" s="15"/>
       <c r="F604" s="15"/>
       <c r="G604" s="15"/>
-      <c r="K604" s="15"/>
+      <c r="K604" s="7"/>
       <c r="L604" s="15"/>
     </row>
     <row r="605" spans="1:15">
       <c r="E605" s="15"/>
       <c r="F605" s="15"/>
       <c r="G605" s="15"/>
-      <c r="K605" s="15"/>
+      <c r="K605" s="7"/>
       <c r="L605" s="15"/>
     </row>
     <row r="606" spans="1:15">
       <c r="E606" s="15"/>
       <c r="F606" s="15"/>
       <c r="G606" s="15"/>
-      <c r="K606" s="15"/>
+      <c r="K606" s="7"/>
       <c r="L606" s="15"/>
     </row>
     <row r="607" spans="1:15">
       <c r="E607" s="15"/>
       <c r="F607" s="15"/>
       <c r="G607" s="15"/>
-      <c r="K607" s="15"/>
+      <c r="K607" s="7"/>
       <c r="L607" s="15"/>
     </row>
     <row r="608" spans="1:15">
       <c r="E608" s="15"/>
       <c r="F608" s="15"/>
       <c r="G608" s="15"/>
-      <c r="K608" s="15"/>
+      <c r="K608" s="7"/>
       <c r="L608" s="15"/>
     </row>
     <row r="609" spans="5:12">
       <c r="E609" s="15"/>
       <c r="F609" s="15"/>
       <c r="G609" s="15"/>
-      <c r="K609" s="15"/>
+      <c r="K609" s="7"/>
       <c r="L609" s="15"/>
+    </row>
+    <row r="610" spans="5:12">
+      <c r="K610" s="7"/>
+    </row>
+    <row r="611" spans="5:12">
+      <c r="K611" s="7"/>
+    </row>
+    <row r="612" spans="5:12">
+      <c r="K612" s="7"/>
+    </row>
+    <row r="613" spans="5:12">
+      <c r="K613" s="7"/>
+    </row>
+    <row r="614" spans="5:12">
+      <c r="K614" s="7"/>
+    </row>
+    <row r="615" spans="5:12">
+      <c r="K615" s="7"/>
+    </row>
+    <row r="616" spans="5:12">
+      <c r="K616" s="7"/>
+    </row>
+    <row r="617" spans="5:12">
+      <c r="K617" s="7"/>
+    </row>
+    <row r="618" spans="5:12">
+      <c r="K618" s="7"/>
+    </row>
+    <row r="619" spans="5:12">
+      <c r="K619" s="7"/>
+    </row>
+    <row r="620" spans="5:12">
+      <c r="K620" s="7"/>
+    </row>
+    <row r="621" spans="5:12">
+      <c r="K621" s="7"/>
+    </row>
+    <row r="622" spans="5:12">
+      <c r="K622" s="7"/>
+    </row>
+    <row r="623" spans="5:12">
+      <c r="K623" s="7"/>
+    </row>
+    <row r="624" spans="5:12">
+      <c r="K624" s="7"/>
+    </row>
+    <row r="625" spans="11:11">
+      <c r="K625" s="7"/>
+    </row>
+    <row r="626" spans="11:11">
+      <c r="K626" s="7"/>
+    </row>
+    <row r="627" spans="11:11">
+      <c r="K627" s="7"/>
+    </row>
+    <row r="628" spans="11:11">
+      <c r="K628" s="7"/>
+    </row>
+    <row r="629" spans="11:11">
+      <c r="K629" s="7"/>
+    </row>
+    <row r="630" spans="11:11">
+      <c r="K630" s="7"/>
+    </row>
+    <row r="631" spans="11:11">
+      <c r="K631" s="7"/>
+    </row>
+    <row r="632" spans="11:11">
+      <c r="K632" s="7"/>
+    </row>
+    <row r="633" spans="11:11">
+      <c r="K633" s="7"/>
+    </row>
+    <row r="634" spans="11:11">
+      <c r="K634" s="7"/>
+    </row>
+    <row r="635" spans="11:11">
+      <c r="K635" s="7"/>
+    </row>
+    <row r="636" spans="11:11">
+      <c r="K636" s="7"/>
+    </row>
+    <row r="637" spans="11:11">
+      <c r="K637" s="7"/>
+    </row>
+    <row r="638" spans="11:11">
+      <c r="K638" s="7"/>
+    </row>
+    <row r="639" spans="11:11">
+      <c r="K639" s="7"/>
+    </row>
+    <row r="640" spans="11:11">
+      <c r="K640" s="7"/>
+    </row>
+    <row r="641" spans="11:11">
+      <c r="K641" s="7"/>
+    </row>
+    <row r="642" spans="11:11">
+      <c r="K642" s="7"/>
+    </row>
+    <row r="643" spans="11:11">
+      <c r="K643" s="7"/>
+    </row>
+    <row r="644" spans="11:11">
+      <c r="K644" s="7"/>
+    </row>
+    <row r="645" spans="11:11">
+      <c r="K645" s="7"/>
+    </row>
+    <row r="646" spans="11:11">
+      <c r="K646" s="7"/>
+    </row>
+    <row r="647" spans="11:11">
+      <c r="K647" s="7"/>
+    </row>
+    <row r="648" spans="11:11">
+      <c r="K648" s="7"/>
+    </row>
+    <row r="649" spans="11:11">
+      <c r="K649" s="7"/>
+    </row>
+    <row r="650" spans="11:11">
+      <c r="K650" s="7"/>
+    </row>
+    <row r="651" spans="11:11">
+      <c r="K651" s="7"/>
+    </row>
+    <row r="652" spans="11:11">
+      <c r="K652" s="7"/>
+    </row>
+    <row r="653" spans="11:11">
+      <c r="K653" s="7"/>
+    </row>
+    <row r="654" spans="11:11">
+      <c r="K654" s="7"/>
+    </row>
+    <row r="655" spans="11:11">
+      <c r="K655" s="7"/>
+    </row>
+    <row r="656" spans="11:11">
+      <c r="K656" s="7"/>
+    </row>
+    <row r="657" spans="11:11">
+      <c r="K657" s="7"/>
+    </row>
+    <row r="658" spans="11:11">
+      <c r="K658" s="7"/>
+    </row>
+    <row r="659" spans="11:11">
+      <c r="K659" s="7"/>
+    </row>
+    <row r="660" spans="11:11">
+      <c r="K660" s="7"/>
+    </row>
+    <row r="661" spans="11:11">
+      <c r="K661" s="7"/>
+    </row>
+    <row r="662" spans="11:11">
+      <c r="K662" s="7"/>
+    </row>
+    <row r="663" spans="11:11">
+      <c r="K663" s="7"/>
+    </row>
+    <row r="664" spans="11:11">
+      <c r="K664" s="7"/>
+    </row>
+    <row r="665" spans="11:11">
+      <c r="K665" s="7"/>
+    </row>
+    <row r="666" spans="11:11">
+      <c r="K666" s="7"/>
+    </row>
+    <row r="667" spans="11:11">
+      <c r="K667" s="7"/>
+    </row>
+    <row r="668" spans="11:11">
+      <c r="K668" s="7"/>
+    </row>
+    <row r="669" spans="11:11">
+      <c r="K669" s="7"/>
+    </row>
+    <row r="670" spans="11:11">
+      <c r="K670" s="7"/>
+    </row>
+    <row r="671" spans="11:11">
+      <c r="K671" s="7"/>
+    </row>
+    <row r="672" spans="11:11">
+      <c r="K672" s="7"/>
+    </row>
+    <row r="673" spans="11:11">
+      <c r="K673" s="7"/>
+    </row>
+    <row r="674" spans="11:11">
+      <c r="K674" s="7"/>
+    </row>
+    <row r="675" spans="11:11">
+      <c r="K675" s="7"/>
+    </row>
+    <row r="676" spans="11:11">
+      <c r="K676" s="7"/>
+    </row>
+    <row r="677" spans="11:11">
+      <c r="K677" s="7"/>
+    </row>
+    <row r="678" spans="11:11">
+      <c r="K678" s="7"/>
+    </row>
+    <row r="679" spans="11:11">
+      <c r="K679" s="7"/>
+    </row>
+    <row r="680" spans="11:11">
+      <c r="K680" s="7"/>
+    </row>
+    <row r="681" spans="11:11">
+      <c r="K681" s="7"/>
+    </row>
+    <row r="682" spans="11:11">
+      <c r="K682" s="7"/>
+    </row>
+    <row r="683" spans="11:11">
+      <c r="K683" s="7"/>
+    </row>
+    <row r="684" spans="11:11">
+      <c r="K684" s="7"/>
+    </row>
+    <row r="685" spans="11:11">
+      <c r="K685" s="7"/>
+    </row>
+    <row r="686" spans="11:11">
+      <c r="K686" s="7"/>
+    </row>
+    <row r="687" spans="11:11">
+      <c r="K687" s="7"/>
+    </row>
+    <row r="689" spans="11:11">
+      <c r="K689" s="15"/>
+    </row>
+    <row r="690" spans="11:11">
+      <c r="K690" s="15"/>
+    </row>
+    <row r="691" spans="11:11">
+      <c r="K691" s="15"/>
+    </row>
+    <row r="692" spans="11:11">
+      <c r="K692" s="15"/>
+    </row>
+    <row r="693" spans="11:11">
+      <c r="K693" s="15"/>
+    </row>
+    <row r="694" spans="11:11">
+      <c r="K694" s="15"/>
+    </row>
+    <row r="695" spans="11:11">
+      <c r="K695" s="15"/>
+    </row>
+    <row r="696" spans="11:11">
+      <c r="K696" s="15"/>
+    </row>
+    <row r="697" spans="11:11">
+      <c r="K697" s="15"/>
+    </row>
+    <row r="698" spans="11:11">
+      <c r="K698" s="15"/>
+    </row>
+    <row r="699" spans="11:11">
+      <c r="K699" s="15"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="6">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="7">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000000000000}">
           <x14:formula1>
             <xm:f>'Drop-down lists'!#REF!</xm:f>
@@ -4798,7 +5107,7 @@
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000001000000}">
           <x14:formula1>
-            <xm:f>'Drop-down lists'!$A$2:$A$12</xm:f>
+            <xm:f>'Drop-down lists'!$A$2:$A$15</xm:f>
           </x14:formula1>
           <xm:sqref>B5</xm:sqref>
         </x14:dataValidation>
@@ -4824,7 +5133,13 @@
           <x14:formula1>
             <xm:f>'Drop-down lists'!$G$2:$G$4</xm:f>
           </x14:formula1>
-          <xm:sqref>K97:K597</xm:sqref>
+          <xm:sqref>K188:K687</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{13AD991D-7B28-F64F-B63A-2495E0FDBD6B}">
+          <x14:formula1>
+            <xm:f>'Drop-down lists'!$G$2:$G$5</xm:f>
+          </x14:formula1>
+          <xm:sqref>K97:K187</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -4835,11 +5150,11 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:H12"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:H15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="29.85546875" customWidth="1"/>
-    <col min="7" max="7" width="11.5703125" customWidth="1"/>
+    <col min="1" max="1" width="29.83203125" customWidth="1"/>
+    <col min="7" max="7" width="11.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
@@ -4867,10 +5182,10 @@
     </row>
     <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="D2" s="3">
         <v>1</v>
@@ -4889,10 +5204,10 @@
       </c>
     </row>
     <row r="3" spans="1:8">
-      <c r="A3" t="s">
+      <c r="A3" s="30" t="s">
         <v>30</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="30" t="s">
         <v>31</v>
       </c>
       <c r="D3" s="3">
@@ -4912,10 +5227,10 @@
       </c>
     </row>
     <row r="4" spans="1:8">
-      <c r="A4" t="s">
+      <c r="A4" s="30" t="s">
         <v>33</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="30" t="s">
         <v>34</v>
       </c>
       <c r="D4" s="3">
@@ -4931,10 +5246,10 @@
       <c r="H4" s="3"/>
     </row>
     <row r="5" spans="1:8">
-      <c r="A5" t="s">
+      <c r="A5" s="30" t="s">
         <v>36</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="30" t="s">
         <v>37</v>
       </c>
       <c r="D5" s="3">
@@ -4944,15 +5259,17 @@
         <v>3</v>
       </c>
       <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
+      <c r="G5" s="3" t="s">
+        <v>163</v>
+      </c>
       <c r="H5" s="3"/>
     </row>
     <row r="6" spans="1:8">
-      <c r="A6" t="s">
-        <v>38</v>
-      </c>
-      <c r="B6" t="s">
-        <v>39</v>
+      <c r="A6" s="31" t="s">
+        <v>164</v>
+      </c>
+      <c r="B6" s="30" t="s">
+        <v>165</v>
       </c>
       <c r="D6" s="3">
         <v>3</v>
@@ -4965,11 +5282,11 @@
       <c r="H6" s="3"/>
     </row>
     <row r="7" spans="1:8">
-      <c r="A7" t="s">
-        <v>40</v>
-      </c>
-      <c r="B7" t="s">
-        <v>41</v>
+      <c r="A7" s="31" t="s">
+        <v>166</v>
+      </c>
+      <c r="B7" s="30" t="s">
+        <v>167</v>
       </c>
       <c r="D7" s="3">
         <v>3.5</v>
@@ -4982,11 +5299,11 @@
       <c r="H7" s="3"/>
     </row>
     <row r="8" spans="1:8">
-      <c r="A8" t="s">
-        <v>42</v>
-      </c>
-      <c r="B8" t="s">
-        <v>43</v>
+      <c r="A8" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="B8" s="30" t="s">
+        <v>39</v>
       </c>
       <c r="D8" s="3">
         <v>4</v>
@@ -4997,11 +5314,11 @@
       <c r="H8" s="3"/>
     </row>
     <row r="9" spans="1:8">
-      <c r="A9" t="s">
-        <v>44</v>
-      </c>
-      <c r="B9" t="s">
-        <v>45</v>
+      <c r="A9" s="30" t="s">
+        <v>168</v>
+      </c>
+      <c r="B9" s="30" t="s">
+        <v>169</v>
       </c>
       <c r="D9" s="3">
         <v>4.5</v>
@@ -5012,11 +5329,11 @@
       <c r="H9" s="3"/>
     </row>
     <row r="10" spans="1:8">
-      <c r="A10" t="s">
-        <v>46</v>
-      </c>
-      <c r="B10" t="s">
-        <v>47</v>
+      <c r="A10" s="30" t="s">
+        <v>170</v>
+      </c>
+      <c r="B10" s="30" t="s">
+        <v>171</v>
       </c>
       <c r="D10" s="3">
         <v>5</v>
@@ -5027,23 +5344,46 @@
       <c r="H10" s="3"/>
     </row>
     <row r="11" spans="1:8">
-      <c r="A11" t="s">
-        <v>48</v>
-      </c>
-      <c r="B11" t="s">
-        <v>49</v>
+      <c r="A11" s="30" t="s">
+        <v>172</v>
+      </c>
+      <c r="B11" s="30" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="12" spans="1:8">
-      <c r="A12" t="s">
-        <v>50</v>
-      </c>
-      <c r="B12" t="s">
-        <v>118</v>
+      <c r="A12" s="30" t="s">
+        <v>40</v>
+      </c>
+      <c r="B12" s="30" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
+      <c r="A13" s="30" t="s">
+        <v>42</v>
+      </c>
+      <c r="B13" s="30" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14" s="30" t="s">
+        <v>44</v>
+      </c>
+      <c r="B14" s="30" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
+      <c r="A15" s="30" t="s">
+        <v>46</v>
+      </c>
+      <c r="B15" s="30" t="s">
+        <v>113</v>
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>